<commit_message>
better neutral art for the characters
</commit_message>
<xml_diff>
--- a/vault/06 Assets/Art Assets.xlsx
+++ b/vault/06 Assets/Art Assets.xlsx
@@ -1262,7 +1262,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>mixed media neutral</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>mixed media neutral</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>mixed media neutral</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>mixed media neutral</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>mixed media neutral</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>placeholder</t>
+          <t>stand-in (neutral)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gui): integrate gold leaf and dark obsidian GUI assets, script updates, and asset tracking
</commit_message>
<xml_diff>
--- a/vault/06 Assets/Art Assets.xlsx
+++ b/vault/06 Assets/Art Assets.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Characters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI &amp; Interface" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2086,4 +2087,464 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DAOCUBATOR / Get Rich Together - GUI &amp; Interface Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mixed-Media &amp; Gold Leaf UI elements matching Asya Abdrahman direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Asset / Component</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Main Menu Title Key Visual</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>game/gui/main_menu.png</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tree of life composed of gold PCB circuits &amp; mycelium roots, hanging ETH tokens, falling sakura petals, and left-side navigation scrim.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Game Menu Background</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>game/gui/game_menu.png</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Atmospheric deep indigo/midnight slate watercolor texture with distressed gold leaf perimeter framing and subtle node watermark for data readability.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NVL Dialogue Background</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>game/gui/nvl.png</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dark atmospheric parchment backing for full-screen narrative scenes.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dialogue Textbox</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>game/gui/textbox.png</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1920x277</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Deep midnight obsidian translucent glass (88% opacity) with 2px gold leaf top trim and decorative gold PCB circuit trace corner brackets.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Character Namebox</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>game/gui/namebox.png</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>450x54</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Raised gold-chamfered plaque with delicate gold circuit pins, 9-slice sliceable for all 6 characters and player.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Choice Button (Idle)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>game/gui/button/choice_idle_background.png</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1185x52</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Semi-transparent dark slate plate with 1px antique gold outline and gold circuit node brackets.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Choice Button (Hover)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>game/gui/button/choice_hover_background.png</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1185x52</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Glowing midnight blue active card with bright gold border, outer gold halo glow, and illuminated gold diamond node chevrons.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Interface Frame (9-slice)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>game/gui/frame.png</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>900x375</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Dual-line gold leaf border with corner PCB pads, used for preferences, save/load, confirm modals, experience select, and lesson popups.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Toast Notification Frame</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>game/gui/notify.png</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1383x64</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Horizontal banner with gold borders and cyan node highlight, used for glossary toasts and top HUD.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fast-Forward Skip Badge</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>game/gui/skip.png</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>360x64</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Compact badge with gold circuit border for skip indicator.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Save/Load Slot Cards</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>game/gui/button/slot_*.png</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>414x309</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Dark card with gold corner pins (idle) and radiant gold border (hover) framing thumbnail saves.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Navigation &amp; Action Buttons</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>game/gui/button/idle_background.png, hover</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>450x49</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Subtle dark slate with fine gold border (idle) and illuminated gold border (hover).</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Checkboxes &amp; Radios</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>game/gui/button/check_*.png, radio_*.png</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>27x49 / 27x64</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Custom gold diamond/check mark boxes and circular gold node radio indicators.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sliders &amp; Scrollbars</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>game/gui/slider/*, scrollbar/*</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Dark groove tracks with polished gold leaf ingot thumbs and subtle gold borders.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Window Icon</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>game/gui/window_icon.png</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>250x250</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Circular medallion with Ethereum crystalline diamond and branching gold circuit nodes on midnight blue.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>mixed media live</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>